<commit_message>
Publish September 7 substitutions and room changes
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -18,12 +18,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
   <si>
     <t>Rok szkolny: 2026/2027</t>
   </si>
   <si>
-    <t>Okres: 01.09.2026 (wt.) - 06.09.2026 (niedz.)</t>
+    <t>Okres: 07.09.2026 (pon.) - 07.09.2026 (pon.)</t>
   </si>
   <si>
     <t>Przeniesiono z</t>
@@ -47,19 +47,19 @@
     <t>Uwagi</t>
   </si>
   <si>
-    <t>02.09.2026, 4, 10:35-11:20, sala: 05</t>
-  </si>
-  <si>
-    <t>02.09.2026, 4, 10:35-11:20, sala: 33</t>
-  </si>
-  <si>
-    <t>Staliś Donata</t>
+    <t>07.09.2026, 1, 08:00-08:45, sala: 05</t>
+  </si>
+  <si>
+    <t>07.09.2026, 1, 08:00-08:45, sala: 2</t>
+  </si>
+  <si>
+    <t>Karczmarz Aleksandra</t>
   </si>
   <si>
     <t>-</t>
   </si>
   <si>
-    <t>4TH|gr1</t>
+    <t>2FC</t>
   </si>
   <si>
     <t>Język angielski</t>
@@ -68,19 +68,49 @@
     <t/>
   </si>
   <si>
-    <t>02.09.2026, 5, 11:25-12:10, sala: 05</t>
-  </si>
-  <si>
-    <t>02.09.2026, 5, 11:25-12:10, sala: 27</t>
-  </si>
-  <si>
-    <t>02.09.2026, 6, 12:25-13:10, sala: 05</t>
-  </si>
-  <si>
-    <t>02.09.2026, 6, 12:25-13:10, sala: 27</t>
-  </si>
-  <si>
-    <t>1FA|gr1</t>
+    <t>07.09.2026, 2, 08:50-09:35, sala: 05</t>
+  </si>
+  <si>
+    <t>07.09.2026, 2, 08:50-09:35, sala: 2</t>
+  </si>
+  <si>
+    <t>2K|gr1</t>
+  </si>
+  <si>
+    <t>07.09.2026, 3, 09:40-10:25, sala: 05</t>
+  </si>
+  <si>
+    <t>07.09.2026, 3, 09:40-10:25, sala: 4</t>
+  </si>
+  <si>
+    <t>2FA</t>
+  </si>
+  <si>
+    <t>07.09.2026, 4, 10:35-11:20, sala: 05</t>
+  </si>
+  <si>
+    <t>07.09.2026, 4, 10:35-11:20, sala: 3</t>
+  </si>
+  <si>
+    <t>2CA</t>
+  </si>
+  <si>
+    <t>07.09.2026, 5, 11:25-12:10, sala: 05</t>
+  </si>
+  <si>
+    <t>07.09.2026, 5, 11:25-12:10, sala: 4</t>
+  </si>
+  <si>
+    <t>2S</t>
+  </si>
+  <si>
+    <t>07.09.2026, 6, 12:25-13:10, sala: 05</t>
+  </si>
+  <si>
+    <t>07.09.2026, 6, 12:25-13:10, sala: 4</t>
+  </si>
+  <si>
+    <t>1TFH|gr1</t>
   </si>
 </sst>
 </file>
@@ -530,7 +560,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{61436d90-ab86-4c99-8a19-5e782c290510}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{40c80021-437c-48f1-8772-fba310692bb5}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -551,12 +581,13 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{3e1545c4-ab5e-4fb3-a21f-7a58f3868f92}">
-  <dimension ref="A1:G4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{438b0631-8cea-4b63-9478-fb1b3490335a}">
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="30.7142857142857" customWidth="1"/>
-    <col min="3" max="3" width="19.4285714285714" customWidth="1"/>
+    <col min="1" max="1" width="30.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="29.7142857142857" customWidth="1"/>
+    <col min="3" max="3" width="20.4285714285714" customWidth="1"/>
     <col min="4" max="4" width="32.7142857142857" customWidth="1"/>
     <col min="5" max="5" width="10.5714285714286" customWidth="1"/>
     <col min="6" max="6" width="14.1428571428571" customWidth="1"/>
@@ -623,7 +654,7 @@
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F3" t="s">
         <v>14</v>
@@ -634,10 +665,10 @@
     </row>
     <row r="4" spans="1:7" ht="15">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
         <v>11</v>
@@ -646,12 +677,81 @@
         <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F4" t="s">
         <v>14</v>
       </c>
       <c r="G4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15">
+      <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15">
+      <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish substitutions for September 7-13
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -23,7 +23,7 @@
     <t>Rok szkolny: 2026/2027</t>
   </si>
   <si>
-    <t>Okres: 07.09.2026 (pon.) - 07.09.2026 (pon.)</t>
+    <t>Okres: 07.09.2026 (pon.) - 13.09.2026 (niedz.)</t>
   </si>
   <si>
     <t>Przeniesiono z</t>
@@ -560,7 +560,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{40c80021-437c-48f1-8772-fba310692bb5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{d06da384-35e2-420d-9596-5e91925e8e1b}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -581,7 +581,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{438b0631-8cea-4b63-9478-fb1b3490335a}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{d8777945-3938-46dc-a1c8-406a9a94c65e}">
   <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Update substitutions and room changes for September 7-13
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -18,12 +18,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="92">
   <si>
     <t>Rok szkolny: 2026/2027</t>
   </si>
   <si>
-    <t>Okres: 07.09.2026 (pon.) - 07.09.2026 (pon.)</t>
+    <t>Okres: 07.09.2026 (pon.) - 13.09.2026 (niedz.)</t>
   </si>
   <si>
     <t>Przeniesiono z</t>
@@ -111,6 +111,189 @@
   </si>
   <si>
     <t>1TFH|gr1</t>
+  </si>
+  <si>
+    <t>08.09.2026, 7, 13:15-14:00, sala: 05</t>
+  </si>
+  <si>
+    <t>08.09.2026, 7, 13:15-14:00, sala: 18</t>
+  </si>
+  <si>
+    <t>Galert Anna</t>
+  </si>
+  <si>
+    <t>1FB</t>
+  </si>
+  <si>
+    <t>Zajęcia z wychowawcą</t>
+  </si>
+  <si>
+    <t>08.09.2026, 8, 14:05-14:50, sala: 05</t>
+  </si>
+  <si>
+    <t>08.09.2026, 8, 14:05-14:50, sala: 18</t>
+  </si>
+  <si>
+    <t>1CA|gr1</t>
+  </si>
+  <si>
+    <t>09.09.2026, 3, 09:40-10:25, sala: 05</t>
+  </si>
+  <si>
+    <t>09.09.2026, 3, 09:40-10:25, sala: 23</t>
+  </si>
+  <si>
+    <t>Granatowska Mariola</t>
+  </si>
+  <si>
+    <t>2K|gr2</t>
+  </si>
+  <si>
+    <t>09.09.2026, 4, 10:35-11:20, sala: 05</t>
+  </si>
+  <si>
+    <t>09.09.2026, 4, 10:35-11:20, sala: 2</t>
+  </si>
+  <si>
+    <t>4TH|gr2</t>
+  </si>
+  <si>
+    <t>09.09.2026, 5, 11:25-12:10, sala: 05</t>
+  </si>
+  <si>
+    <t>09.09.2026, 5, 11:25-12:10, sala: bib</t>
+  </si>
+  <si>
+    <t>09.09.2026, 6, 12:25-13:10, sala: 05</t>
+  </si>
+  <si>
+    <t>09.09.2026, 6, 12:25-13:10, sala: 2</t>
+  </si>
+  <si>
+    <t>3TFA</t>
+  </si>
+  <si>
+    <t>09.09.2026, 7, 13:15-14:00, sala: 05</t>
+  </si>
+  <si>
+    <t>09.09.2026, 7, 13:15-14:00, sala: 2</t>
+  </si>
+  <si>
+    <t>2CB</t>
+  </si>
+  <si>
+    <t>10.09.2026, 3, 09:40-10:25, sala: 05</t>
+  </si>
+  <si>
+    <t>10.09.2026, 3, 09:40-10:25, sala: 3</t>
+  </si>
+  <si>
+    <t>1FA|gr2</t>
+  </si>
+  <si>
+    <t>10.09.2026, 4, 10:35-11:20, sala: 05</t>
+  </si>
+  <si>
+    <t>10.09.2026, 4, 10:35-11:20, sala: 3</t>
+  </si>
+  <si>
+    <t>1K|gr1</t>
+  </si>
+  <si>
+    <t>10.09.2026, 5, 11:25-12:10, sala: 05</t>
+  </si>
+  <si>
+    <t>10.09.2026, 5, 11:25-12:10, sala: 3</t>
+  </si>
+  <si>
+    <t>1FC|gr1</t>
+  </si>
+  <si>
+    <t>10.09.2026, 6, 12:25-13:10, sala: 05</t>
+  </si>
+  <si>
+    <t>10.09.2026, 6, 12:25-13:10, sala: 3</t>
+  </si>
+  <si>
+    <t>1TFA|gr2</t>
+  </si>
+  <si>
+    <t>10.09.2026, 7, 13:15-14:00, sala: 05</t>
+  </si>
+  <si>
+    <t>10.09.2026, 7, 13:15-14:00, sala: 5</t>
+  </si>
+  <si>
+    <t>1S|gr2</t>
+  </si>
+  <si>
+    <t>11.09.2026, 2, 08:50-09:35, sala: 05</t>
+  </si>
+  <si>
+    <t>11.09.2026, 2, 08:50-09:35, sala: 18</t>
+  </si>
+  <si>
+    <t>4TFA</t>
+  </si>
+  <si>
+    <t>11.09.2026, 3, 09:40-10:25, sala: 05</t>
+  </si>
+  <si>
+    <t>11.09.2026, 3, 09:40-10:25, sala: 17</t>
+  </si>
+  <si>
+    <t>11.09.2026, 4, 10:35-11:20, sala: 05</t>
+  </si>
+  <si>
+    <t>11.09.2026, 4, 10:35-11:20, sala: 17</t>
+  </si>
+  <si>
+    <t>11.09.2026, 5, 11:25-12:10, sala: 05</t>
+  </si>
+  <si>
+    <t>11.09.2026, 5, 11:25-12:10, sala: 40</t>
+  </si>
+  <si>
+    <t>1TFB|gr1</t>
+  </si>
+  <si>
+    <t>11.09.2026, 6, 12:25-13:10, sala: 05</t>
+  </si>
+  <si>
+    <t>11.09.2026, 6, 12:25-13:10, sala: 40</t>
+  </si>
+  <si>
+    <t>3TFB|gr1</t>
+  </si>
+  <si>
+    <t>11.09.2026, 7, 13:15-14:00, sala: 05</t>
+  </si>
+  <si>
+    <t>11.09.2026, 7, 13:15-14:00, sala: 41</t>
+  </si>
+  <si>
+    <t>1CB|gr1</t>
+  </si>
+  <si>
+    <t>11.09.2026, 8, 14:05-14:50, sala: 05</t>
+  </si>
+  <si>
+    <t>11.09.2026, 8, 14:05-14:50, sala: 40</t>
+  </si>
+  <si>
+    <t>11.09.2026, 9, 14:55-15:40, sala: 05</t>
+  </si>
+  <si>
+    <t>11.09.2026, 9, 14:55-15:40, sala: 40</t>
+  </si>
+  <si>
+    <t>11.09.2026, 10, 15:45-16:30, sala: 05</t>
+  </si>
+  <si>
+    <t>11.09.2026, 10, 15:45-16:30, sala: 40</t>
+  </si>
+  <si>
+    <t>1FB|gr1</t>
   </si>
 </sst>
 </file>
@@ -560,7 +743,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{40c80021-437c-48f1-8772-fba310692bb5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{5d64cdcb-b1f1-43c1-bc68-85d26f780813}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -581,16 +764,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{438b0631-8cea-4b63-9478-fb1b3490335a}">
-  <dimension ref="A1:G7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{b07396a0-dd9b-4d91-86bc-f0cb21bca76a}">
+  <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="30.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="29.7142857142857" customWidth="1"/>
+    <col min="1" max="2" width="31.7142857142857" customWidth="1"/>
     <col min="3" max="3" width="20.4285714285714" customWidth="1"/>
     <col min="4" max="4" width="32.7142857142857" customWidth="1"/>
     <col min="5" max="5" width="10.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="14.1428571428571" customWidth="1"/>
+    <col min="6" max="6" width="20.7142857142857" customWidth="1"/>
     <col min="7" max="7" width="9.28571428571429" customWidth="1"/>
   </cols>
   <sheetData>
@@ -755,6 +937,489 @@
         <v>15</v>
       </c>
     </row>
+    <row r="8" spans="1:7" ht="15">
+      <c r="A8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" t="s">
+        <v>35</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15">
+      <c r="A9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15">
+      <c r="A10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s">
+        <v>42</v>
+      </c>
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15">
+      <c r="A11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15">
+      <c r="A12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" t="s">
+        <v>45</v>
+      </c>
+      <c r="F12" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15">
+      <c r="A13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15">
+      <c r="A14" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" t="s">
+        <v>53</v>
+      </c>
+      <c r="F14" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15">
+      <c r="A15" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" t="s">
+        <v>33</v>
+      </c>
+      <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" t="s">
+        <v>56</v>
+      </c>
+      <c r="F15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="15">
+      <c r="A16" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" t="s">
+        <v>33</v>
+      </c>
+      <c r="D16" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" t="s">
+        <v>59</v>
+      </c>
+      <c r="F16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="15">
+      <c r="A17" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" t="s">
+        <v>62</v>
+      </c>
+      <c r="F17" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="15">
+      <c r="A18" t="s">
+        <v>63</v>
+      </c>
+      <c r="B18" t="s">
+        <v>64</v>
+      </c>
+      <c r="C18" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" t="s">
+        <v>65</v>
+      </c>
+      <c r="F18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="15">
+      <c r="A19" t="s">
+        <v>66</v>
+      </c>
+      <c r="B19" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" t="s">
+        <v>33</v>
+      </c>
+      <c r="D19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" t="s">
+        <v>68</v>
+      </c>
+      <c r="F19" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="15">
+      <c r="A20" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" t="s">
+        <v>33</v>
+      </c>
+      <c r="D20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" t="s">
+        <v>71</v>
+      </c>
+      <c r="F20" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="15">
+      <c r="A21" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" t="s">
+        <v>73</v>
+      </c>
+      <c r="C21" t="s">
+        <v>33</v>
+      </c>
+      <c r="D21" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" t="s">
+        <v>71</v>
+      </c>
+      <c r="F21" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="15">
+      <c r="A22" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" t="s">
+        <v>75</v>
+      </c>
+      <c r="C22" t="s">
+        <v>33</v>
+      </c>
+      <c r="D22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" t="s">
+        <v>68</v>
+      </c>
+      <c r="F22" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15">
+      <c r="A23" t="s">
+        <v>76</v>
+      </c>
+      <c r="B23" t="s">
+        <v>77</v>
+      </c>
+      <c r="C23" t="s">
+        <v>33</v>
+      </c>
+      <c r="D23" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" t="s">
+        <v>78</v>
+      </c>
+      <c r="F23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15">
+      <c r="A24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B24" t="s">
+        <v>80</v>
+      </c>
+      <c r="C24" t="s">
+        <v>33</v>
+      </c>
+      <c r="D24" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F24" t="s">
+        <v>14</v>
+      </c>
+      <c r="G24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="15">
+      <c r="A25" t="s">
+        <v>82</v>
+      </c>
+      <c r="B25" t="s">
+        <v>83</v>
+      </c>
+      <c r="C25" t="s">
+        <v>33</v>
+      </c>
+      <c r="D25" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" t="s">
+        <v>84</v>
+      </c>
+      <c r="F25" t="s">
+        <v>14</v>
+      </c>
+      <c r="G25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="15">
+      <c r="A26" t="s">
+        <v>85</v>
+      </c>
+      <c r="B26" t="s">
+        <v>86</v>
+      </c>
+      <c r="C26" t="s">
+        <v>33</v>
+      </c>
+      <c r="D26" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" t="s">
+        <v>59</v>
+      </c>
+      <c r="F26" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="15">
+      <c r="A27" t="s">
+        <v>87</v>
+      </c>
+      <c r="B27" t="s">
+        <v>88</v>
+      </c>
+      <c r="C27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D27" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" t="s">
+        <v>62</v>
+      </c>
+      <c r="F27" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="15">
+      <c r="A28" t="s">
+        <v>89</v>
+      </c>
+      <c r="B28" t="s">
+        <v>90</v>
+      </c>
+      <c r="C28" t="s">
+        <v>33</v>
+      </c>
+      <c r="D28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" t="s">
+        <v>91</v>
+      </c>
+      <c r="F28" t="s">
+        <v>14</v>
+      </c>
+      <c r="G28" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Prepare production release with current changes and automatic interface refresh
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="92">
   <si>
     <t>Rok szkolny: 2026/2027</t>
   </si>
@@ -111,6 +111,189 @@
   </si>
   <si>
     <t>1TFH|gr1</t>
+  </si>
+  <si>
+    <t>08.09.2026, 7, 13:15-14:00, sala: 05</t>
+  </si>
+  <si>
+    <t>08.09.2026, 7, 13:15-14:00, sala: 18</t>
+  </si>
+  <si>
+    <t>Galert Anna</t>
+  </si>
+  <si>
+    <t>1FB</t>
+  </si>
+  <si>
+    <t>Zajęcia z wychowawcą</t>
+  </si>
+  <si>
+    <t>08.09.2026, 8, 14:05-14:50, sala: 05</t>
+  </si>
+  <si>
+    <t>08.09.2026, 8, 14:05-14:50, sala: 18</t>
+  </si>
+  <si>
+    <t>1CA|gr1</t>
+  </si>
+  <si>
+    <t>09.09.2026, 3, 09:40-10:25, sala: 05</t>
+  </si>
+  <si>
+    <t>09.09.2026, 3, 09:40-10:25, sala: 23</t>
+  </si>
+  <si>
+    <t>Granatowska Mariola</t>
+  </si>
+  <si>
+    <t>2K|gr2</t>
+  </si>
+  <si>
+    <t>09.09.2026, 4, 10:35-11:20, sala: 05</t>
+  </si>
+  <si>
+    <t>09.09.2026, 4, 10:35-11:20, sala: 2</t>
+  </si>
+  <si>
+    <t>4TH|gr2</t>
+  </si>
+  <si>
+    <t>09.09.2026, 5, 11:25-12:10, sala: 05</t>
+  </si>
+  <si>
+    <t>09.09.2026, 5, 11:25-12:10, sala: bib</t>
+  </si>
+  <si>
+    <t>09.09.2026, 6, 12:25-13:10, sala: 05</t>
+  </si>
+  <si>
+    <t>09.09.2026, 6, 12:25-13:10, sala: 2</t>
+  </si>
+  <si>
+    <t>3TFA</t>
+  </si>
+  <si>
+    <t>09.09.2026, 7, 13:15-14:00, sala: 05</t>
+  </si>
+  <si>
+    <t>09.09.2026, 7, 13:15-14:00, sala: 2</t>
+  </si>
+  <si>
+    <t>2CB</t>
+  </si>
+  <si>
+    <t>10.09.2026, 3, 09:40-10:25, sala: 05</t>
+  </si>
+  <si>
+    <t>10.09.2026, 3, 09:40-10:25, sala: 3</t>
+  </si>
+  <si>
+    <t>1FA|gr2</t>
+  </si>
+  <si>
+    <t>10.09.2026, 4, 10:35-11:20, sala: 05</t>
+  </si>
+  <si>
+    <t>10.09.2026, 4, 10:35-11:20, sala: 3</t>
+  </si>
+  <si>
+    <t>1K|gr1</t>
+  </si>
+  <si>
+    <t>10.09.2026, 5, 11:25-12:10, sala: 05</t>
+  </si>
+  <si>
+    <t>10.09.2026, 5, 11:25-12:10, sala: 3</t>
+  </si>
+  <si>
+    <t>1FC|gr1</t>
+  </si>
+  <si>
+    <t>10.09.2026, 6, 12:25-13:10, sala: 05</t>
+  </si>
+  <si>
+    <t>10.09.2026, 6, 12:25-13:10, sala: 3</t>
+  </si>
+  <si>
+    <t>1TFA|gr2</t>
+  </si>
+  <si>
+    <t>10.09.2026, 7, 13:15-14:00, sala: 05</t>
+  </si>
+  <si>
+    <t>10.09.2026, 7, 13:15-14:00, sala: 5</t>
+  </si>
+  <si>
+    <t>1S|gr2</t>
+  </si>
+  <si>
+    <t>11.09.2026, 2, 08:50-09:35, sala: 05</t>
+  </si>
+  <si>
+    <t>11.09.2026, 2, 08:50-09:35, sala: 18</t>
+  </si>
+  <si>
+    <t>4TFA</t>
+  </si>
+  <si>
+    <t>11.09.2026, 3, 09:40-10:25, sala: 05</t>
+  </si>
+  <si>
+    <t>11.09.2026, 3, 09:40-10:25, sala: 17</t>
+  </si>
+  <si>
+    <t>11.09.2026, 4, 10:35-11:20, sala: 05</t>
+  </si>
+  <si>
+    <t>11.09.2026, 4, 10:35-11:20, sala: 17</t>
+  </si>
+  <si>
+    <t>11.09.2026, 5, 11:25-12:10, sala: 05</t>
+  </si>
+  <si>
+    <t>11.09.2026, 5, 11:25-12:10, sala: 40</t>
+  </si>
+  <si>
+    <t>1TFB|gr1</t>
+  </si>
+  <si>
+    <t>11.09.2026, 6, 12:25-13:10, sala: 05</t>
+  </si>
+  <si>
+    <t>11.09.2026, 6, 12:25-13:10, sala: 40</t>
+  </si>
+  <si>
+    <t>3TFB|gr1</t>
+  </si>
+  <si>
+    <t>11.09.2026, 7, 13:15-14:00, sala: 05</t>
+  </si>
+  <si>
+    <t>11.09.2026, 7, 13:15-14:00, sala: 41</t>
+  </si>
+  <si>
+    <t>1CB|gr1</t>
+  </si>
+  <si>
+    <t>11.09.2026, 8, 14:05-14:50, sala: 05</t>
+  </si>
+  <si>
+    <t>11.09.2026, 8, 14:05-14:50, sala: 40</t>
+  </si>
+  <si>
+    <t>11.09.2026, 9, 14:55-15:40, sala: 05</t>
+  </si>
+  <si>
+    <t>11.09.2026, 9, 14:55-15:40, sala: 40</t>
+  </si>
+  <si>
+    <t>11.09.2026, 10, 15:45-16:30, sala: 05</t>
+  </si>
+  <si>
+    <t>11.09.2026, 10, 15:45-16:30, sala: 40</t>
+  </si>
+  <si>
+    <t>1FB|gr1</t>
   </si>
 </sst>
 </file>
@@ -560,7 +743,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{d06da384-35e2-420d-9596-5e91925e8e1b}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{5d64cdcb-b1f1-43c1-bc68-85d26f780813}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -581,16 +764,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{d8777945-3938-46dc-a1c8-406a9a94c65e}">
-  <dimension ref="A1:G7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{b07396a0-dd9b-4d91-86bc-f0cb21bca76a}">
+  <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="30.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="29.7142857142857" customWidth="1"/>
+    <col min="1" max="2" width="31.7142857142857" customWidth="1"/>
     <col min="3" max="3" width="20.4285714285714" customWidth="1"/>
     <col min="4" max="4" width="32.7142857142857" customWidth="1"/>
     <col min="5" max="5" width="10.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="14.1428571428571" customWidth="1"/>
+    <col min="6" max="6" width="20.7142857142857" customWidth="1"/>
     <col min="7" max="7" width="9.28571428571429" customWidth="1"/>
   </cols>
   <sheetData>
@@ -755,6 +937,489 @@
         <v>15</v>
       </c>
     </row>
+    <row r="8" spans="1:7" ht="15">
+      <c r="A8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" t="s">
+        <v>35</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15">
+      <c r="A9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15">
+      <c r="A10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s">
+        <v>42</v>
+      </c>
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15">
+      <c r="A11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15">
+      <c r="A12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" t="s">
+        <v>45</v>
+      </c>
+      <c r="F12" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15">
+      <c r="A13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15">
+      <c r="A14" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" t="s">
+        <v>53</v>
+      </c>
+      <c r="F14" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15">
+      <c r="A15" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" t="s">
+        <v>33</v>
+      </c>
+      <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" t="s">
+        <v>56</v>
+      </c>
+      <c r="F15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="15">
+      <c r="A16" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" t="s">
+        <v>33</v>
+      </c>
+      <c r="D16" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" t="s">
+        <v>59</v>
+      </c>
+      <c r="F16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="15">
+      <c r="A17" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" t="s">
+        <v>62</v>
+      </c>
+      <c r="F17" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="15">
+      <c r="A18" t="s">
+        <v>63</v>
+      </c>
+      <c r="B18" t="s">
+        <v>64</v>
+      </c>
+      <c r="C18" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" t="s">
+        <v>65</v>
+      </c>
+      <c r="F18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="15">
+      <c r="A19" t="s">
+        <v>66</v>
+      </c>
+      <c r="B19" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" t="s">
+        <v>33</v>
+      </c>
+      <c r="D19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" t="s">
+        <v>68</v>
+      </c>
+      <c r="F19" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="15">
+      <c r="A20" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" t="s">
+        <v>33</v>
+      </c>
+      <c r="D20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" t="s">
+        <v>71</v>
+      </c>
+      <c r="F20" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="15">
+      <c r="A21" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" t="s">
+        <v>73</v>
+      </c>
+      <c r="C21" t="s">
+        <v>33</v>
+      </c>
+      <c r="D21" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" t="s">
+        <v>71</v>
+      </c>
+      <c r="F21" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="15">
+      <c r="A22" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" t="s">
+        <v>75</v>
+      </c>
+      <c r="C22" t="s">
+        <v>33</v>
+      </c>
+      <c r="D22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" t="s">
+        <v>68</v>
+      </c>
+      <c r="F22" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15">
+      <c r="A23" t="s">
+        <v>76</v>
+      </c>
+      <c r="B23" t="s">
+        <v>77</v>
+      </c>
+      <c r="C23" t="s">
+        <v>33</v>
+      </c>
+      <c r="D23" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" t="s">
+        <v>78</v>
+      </c>
+      <c r="F23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15">
+      <c r="A24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B24" t="s">
+        <v>80</v>
+      </c>
+      <c r="C24" t="s">
+        <v>33</v>
+      </c>
+      <c r="D24" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F24" t="s">
+        <v>14</v>
+      </c>
+      <c r="G24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="15">
+      <c r="A25" t="s">
+        <v>82</v>
+      </c>
+      <c r="B25" t="s">
+        <v>83</v>
+      </c>
+      <c r="C25" t="s">
+        <v>33</v>
+      </c>
+      <c r="D25" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" t="s">
+        <v>84</v>
+      </c>
+      <c r="F25" t="s">
+        <v>14</v>
+      </c>
+      <c r="G25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="15">
+      <c r="A26" t="s">
+        <v>85</v>
+      </c>
+      <c r="B26" t="s">
+        <v>86</v>
+      </c>
+      <c r="C26" t="s">
+        <v>33</v>
+      </c>
+      <c r="D26" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" t="s">
+        <v>59</v>
+      </c>
+      <c r="F26" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="15">
+      <c r="A27" t="s">
+        <v>87</v>
+      </c>
+      <c r="B27" t="s">
+        <v>88</v>
+      </c>
+      <c r="C27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D27" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" t="s">
+        <v>62</v>
+      </c>
+      <c r="F27" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="15">
+      <c r="A28" t="s">
+        <v>89</v>
+      </c>
+      <c r="B28" t="s">
+        <v>90</v>
+      </c>
+      <c r="C28" t="s">
+        <v>33</v>
+      </c>
+      <c r="D28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" t="s">
+        <v>91</v>
+      </c>
+      <c r="F28" t="s">
+        <v>14</v>
+      </c>
+      <c r="G28" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update substitutions and transfers for September 7–13
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -743,7 +743,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{5d64cdcb-b1f1-43c1-bc68-85d26f780813}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{569de468-be56-4b9c-b8e8-5f25a1b9f03e}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -764,7 +764,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{b07396a0-dd9b-4d91-86bc-f0cb21bca76a}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{a951eef4-1939-47f3-9368-c1732cb7c658}">
   <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>

</xml_diff>